<commit_message>
Bandeau de campagne sur tout le site
Rail vertical a droite sur grand ecran, barre en bas sur mobile : logo,
pourcentage, accroche, compte a rebours, bouton et code.

Aucune donnee de firme dans le composant. lib/campagne.ts choisit parmi
les fiches l'offre confirmee dont la date de fin est encore a venir, la
plus forte remise d'abord. Une offre permanente n'y entre pas : un compte
a rebours sans echeance n'a pas de sens.

Le bandeau se retire seul a l'expiration, meme onglet ouvert, et le
visiteur peut le fermer pour 24 heures.

Nouvelle colonne generique « accroche » dans l'onglet Offre, pour dire ce
que la campagne donne en plus du pourcentage.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MODELE-propfirm.xlsx
+++ b/MODELE-propfirm.xlsx
@@ -1314,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1484,6 +1484,18 @@
       <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Seule une offre confirmed s'affiche : remise, code, Copy code et Claim deal. Vide ou needs_confirmation : la carte garde le plan, le prix public et Continue to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>accroche</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Une phrase courte pour le bandeau de campagne du site : ce que l'offre donne, en plus du pourcentage. Vide : le bandeau n'affiche que la remise.</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4064,9 +4076,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Une offre peut valoir plus que son pourcentage : le bonus se voit
Demande d'Eva Saint-Arroman (affiliation Earn2Trade, 29/09) : le reset offert
doit se voir sur /compare et sur la fiche, pas se lire en petit.

Nouveau champ « bonus » dans l'onglet Offre du modele — deux ou trois mots,
« +1 free reset » pour Earn2Trade. Il s'affiche en pastille pleine :
  - fiche : sous le pourcentage, au meme poids visuel ;
  - /compare : dans le cadre promo en vue grille, a cote du taux en vue liste.

Generique : une firme sans bonus n'affiche rien, et le bonus suit la campagne
— il disparait avec elle, comme l'accroche.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MODELE-propfirm.xlsx
+++ b/MODELE-propfirm.xlsx
@@ -1314,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1520,6 +1520,18 @@
       <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Fin de la campagne, date et heure ISO. Passee, le taux de campagne et l'accroche disparaissent, l'offre permanente reste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>bonus</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Deux ou trois mots pour ce que l'offre donne en plus du pourcentage (« +1 free reset »). Affiche en pastille sur la fiche et sur la carte /compare. Suit la campagne : il disparait avec elle.</t>
         </is>
       </c>
     </row>

</xml_diff>